<commit_message>
Enhance curriculum upload to verify member and include registrant info
Adds registrant information extraction from Excel, member verification API, and improves curriculum data handling in admin.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: c50f358d-2aa3-4eab-8973-75a668fc9620
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/8f9bc033-6ae0-4fd7-95cb-7a6faad7f5f8/452d16f5-bfc5-428f-b032-7888425d3320.jpg
</commit_message>
<xml_diff>
--- a/public/uploads/test-curriculum-sample.xlsx
+++ b/public/uploads/test-curriculum-sample.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:G21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -411,169 +411,234 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>제목</v>
-      </c>
-      <c r="B3" t="str">
-        <v>반려동물 재활 전문 과정</v>
+        <v>== 등록자 정보 ==</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>설명</v>
+        <v>등록자명</v>
       </c>
       <c r="B4" t="str">
-        <v>반려동물의 재활과 회복을 위한 전문적인 교육 과정입니다.</v>
+        <v>김훈련사</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>카테고리</v>
+        <v>등록자 이메일</v>
       </c>
       <c r="B5" t="str">
-        <v>재활훈련</v>
+        <v>trainer@example.com</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>전체가격</v>
+        <v>등록자 전화번호</v>
       </c>
       <c r="B6" t="str">
-        <v>400000</v>
+        <v>010-1234-5678</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v>소속기관</v>
+      </c>
+      <c r="B7" t="str">
+        <v>테일즈 훈련센터</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>강의 구성</v>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>회차</v>
-      </c>
-      <c r="B9" t="str">
-        <v>강의명</v>
-      </c>
-      <c r="C9" t="str">
-        <v>설명</v>
-      </c>
-      <c r="D9" t="str">
-        <v>시간(분)</v>
-      </c>
-      <c r="E9" t="str">
-        <v>무료여부</v>
-      </c>
-      <c r="F9" t="str">
-        <v>개별가격</v>
+        <v>== 커리큘럼 기본정보 ==</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>1</v>
+        <v>제목</v>
       </c>
       <c r="B10" t="str">
-        <v>재활 기초 평가</v>
-      </c>
-      <c r="C10" t="str">
-        <v>반려동물의 신체 상태 평가 및 재활 계획 수립</v>
-      </c>
-      <c r="D10" t="str">
-        <v>90</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Y</v>
-      </c>
-      <c r="F10" t="str">
-        <v>0</v>
+        <v>반려동물 재활 전문 과정</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2</v>
+        <v>설명</v>
       </c>
       <c r="B11" t="str">
-        <v>기초 운동치료</v>
-      </c>
-      <c r="C11" t="str">
-        <v>기본적인 물리치료 및 운동요법</v>
-      </c>
-      <c r="D11" t="str">
-        <v>60</v>
-      </c>
-      <c r="E11" t="str">
-        <v>N</v>
-      </c>
-      <c r="F11" t="str">
-        <v>100000</v>
+        <v>반려동물의 재활과 회복을 위한 전문적인 교육 과정입니다.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>3</v>
+        <v>카테고리</v>
       </c>
       <c r="B12" t="str">
-        <v>전문 재활 운동</v>
-      </c>
-      <c r="C12" t="str">
-        <v>맞춤형 재활 운동 프로그램</v>
-      </c>
-      <c r="D12" t="str">
-        <v>120</v>
-      </c>
-      <c r="E12" t="str">
-        <v>N</v>
-      </c>
-      <c r="F12" t="str">
-        <v>150000</v>
+        <v>재활훈련</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>4</v>
+        <v>전체가격</v>
       </c>
       <c r="B13" t="str">
-        <v>재활 효과 평가</v>
-      </c>
-      <c r="C13" t="str">
-        <v>재활 진행 상황 평가 및 조정</v>
-      </c>
-      <c r="D13" t="str">
-        <v>90</v>
-      </c>
-      <c r="E13" t="str">
-        <v>N</v>
-      </c>
-      <c r="F13" t="str">
-        <v>100000</v>
+        <v>400000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>== 강의 구성 ==</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>회차</v>
+      </c>
+      <c r="B16" t="str">
+        <v>강의명</v>
+      </c>
+      <c r="C16" t="str">
+        <v>설명</v>
+      </c>
+      <c r="D16" t="str">
+        <v>시간(분)</v>
+      </c>
+      <c r="E16" t="str">
+        <v>무료여부</v>
+      </c>
+      <c r="F16" t="str">
+        <v>개별가격</v>
+      </c>
+      <c r="G16" t="str">
+        <v>준비물</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>1</v>
+      </c>
+      <c r="B17" t="str">
+        <v>재활 기초 평가</v>
+      </c>
+      <c r="C17" t="str">
+        <v>반려동물의 신체 상태 평가 및 재활 계획 수립</v>
+      </c>
+      <c r="D17" t="str">
+        <v>90</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Y</v>
+      </c>
+      <c r="F17" t="str">
+        <v>0</v>
+      </c>
+      <c r="G17" t="str">
+        <v>체크리스트, 평가지, 줄자</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>2</v>
+      </c>
+      <c r="B18" t="str">
+        <v>기초 운동치료</v>
+      </c>
+      <c r="C18" t="str">
+        <v>기본적인 물리치료 및 운동요법</v>
+      </c>
+      <c r="D18" t="str">
+        <v>60</v>
+      </c>
+      <c r="E18" t="str">
+        <v>N</v>
+      </c>
+      <c r="F18" t="str">
+        <v>100000</v>
+      </c>
+      <c r="G18" t="str">
+        <v>운동 매트, 간식, 장난감</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>3</v>
+      </c>
+      <c r="B19" t="str">
+        <v>전문 재활 운동</v>
+      </c>
+      <c r="C19" t="str">
+        <v>맞춤형 재활 운동 프로그램</v>
+      </c>
+      <c r="D19" t="str">
+        <v>120</v>
+      </c>
+      <c r="E19" t="str">
+        <v>N</v>
+      </c>
+      <c r="F19" t="str">
+        <v>150000</v>
+      </c>
+      <c r="G19" t="str">
+        <v>재활 도구, 밸런스 볼, 슬링</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>4</v>
+      </c>
+      <c r="B20" t="str">
+        <v>재활 효과 평가</v>
+      </c>
+      <c r="C20" t="str">
+        <v>재활 진행 상황 평가 및 조정</v>
+      </c>
+      <c r="D20" t="str">
+        <v>90</v>
+      </c>
+      <c r="E20" t="str">
+        <v>N</v>
+      </c>
+      <c r="F20" t="str">
+        <v>100000</v>
+      </c>
+      <c r="G20" t="str">
+        <v>재평가 도구, 측정 기구</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
         <v>5</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B21" t="str">
         <v>가정 관리 교육</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C21" t="str">
         <v>집에서 할 수 있는 관리 방법</v>
       </c>
-      <c r="D14" t="str">
+      <c r="D21" t="str">
         <v>60</v>
       </c>
-      <c r="E14" t="str">
+      <c r="E21" t="str">
         <v>N</v>
       </c>
-      <c r="F14" t="str">
+      <c r="F21" t="str">
         <v>50000</v>
+      </c>
+      <c r="G21" t="str">
+        <v>홈케어 가이드, 운동 도구</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>